<commit_message>
Update 2.Cálculo KNN y decisión.xlsx
</commit_message>
<xml_diff>
--- a/2.Data Preparation ML Loan Approval Financial Institution/Fundaments/2.Cálculo KNN y decisión.xlsx
+++ b/2.Data Preparation ML Loan Approval Financial Institution/Fundaments/2.Cálculo KNN y decisión.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\9.Docencia\1.MATERIAS\2.IA y ML\2.PRÁCTICAS\Práctica2. KNN Transformación y Selección de Variables\GUIA RECURSOS Y RUBRICA - PRACTICA 2 KNN TRANSFORMACION SELECCION VARIABLES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhurtadoo\Proyectos\MachineLearning-Engineering-Production-Portfolio\2.Data Preparation ML Loan Approval Financial Institution\Fundaments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534AC151-5278-48B3-ABE3-FBFCD4EFFD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690154BB-9761-4D69-B992-6184561524FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>2. Identificar los K vecinos</t>
   </si>
@@ -108,6 +108,12 @@
   </si>
   <si>
     <t>media costo:</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>c1-c3:</t>
   </si>
 </sst>
 </file>
@@ -625,8 +631,8 @@
       <c r="D2" s="3">
         <v>250</v>
       </c>
-      <c r="E2" s="8">
-        <v>60000</v>
+      <c r="E2" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="H2" t="s">
         <v>2</v>
@@ -648,8 +654,8 @@
       <c r="D3" s="3">
         <v>300</v>
       </c>
-      <c r="E3" s="4">
-        <v>75000</v>
+      <c r="E3" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H3" t="s">
         <v>0</v>
@@ -791,6 +797,25 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13">
+        <f>(B2-B4)^2</f>
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <f>(C2-C4)^2</f>
+        <v>2500</v>
+      </c>
+      <c r="D13">
+        <f>(D2-D4)^2</f>
+        <v>4900</v>
+      </c>
+      <c r="E13">
+        <f>SQRT(SUM(B13:D13))</f>
+        <v>86.046499057195817</v>
+      </c>
       <c r="L13" s="1" t="s">
         <v>4</v>
       </c>

</xml_diff>